<commit_message>
docs(scrum): incorporar documentos del Sprint 5 y actualizar Product Backlog
- Añadir registros de reuniones diarias, retrospectiva y Sprint Backlog.
- Actualizar estados, iteraciones y comentarios del Product Backlog según el avance implementado.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Documentación/Product Backlog SIGET.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Documentación/Product Backlog SIGET.xlsx
@@ -1,40 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Historias de Usuario" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Instructivo" sheetId="2" r:id="rId5"/>
+    <sheet name="Historias de Usuario" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructivo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
   <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="q2nriHmzllqOlEG5zIeVK4lWva3CuMvxgo1L19IBFvk="/>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
   <si>
-    <t>Desarrollo ágil: Pila de Producto (Product Backlog)</t>
+    <t xml:space="preserve">Desarrollo ágil: Pila de Producto (Product Backlog)</t>
   </si>
   <si>
-    <t>Pila de Producto (Product Backlog): Instructivo</t>
+    <t xml:space="preserve">Tabla ordenada por Iteración (Sprint)</t>
   </si>
   <si>
-    <t>Tabla ordenada por Iteración (Sprint)</t>
+    <t xml:space="preserve">Identificador (ID) de la Historia</t>
   </si>
   <si>
-    <t>Elaborado por: pmoinformatica.com</t>
-  </si>
-  <si>
-    <t>Identificador (ID) de la Historia</t>
-  </si>
-  <si>
-    <t>Enunciado de la Historia</t>
+    <t xml:space="preserve">Enunciado de la Historia</t>
   </si>
   <si>
     <t>Alias</t>
@@ -43,49 +37,433 @@
     <t>Estado</t>
   </si>
   <si>
-    <t>Dimensión / Esfuerzo</t>
+    <t xml:space="preserve">Dimensión / Esfuerzo</t>
   </si>
   <si>
-    <t>Iteración (Sprint)</t>
+    <t xml:space="preserve">Iteración (Sprint)</t>
   </si>
   <si>
     <t>Prioridad</t>
   </si>
   <si>
-    <t>Columna</t>
+    <t>Comentarios</t>
   </si>
   <si>
-    <t>Comentarios</t>
+    <t>E1-H1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario de SIGET, necesito iniciar sesión en el sistema mediante el proveedor externo de identidad, con la finalidad de acceder a las funcionalidades autorizadas según mi rol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iniciar sesión</t>
+  </si>
+  <si>
+    <t>Hecho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inicio y cierre de sesión implementados y validados manualmente. El acceso aplica los roles y permisos locales.</t>
+  </si>
+  <si>
+    <t>E1-H2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario de SIGET, necesito recuperar el acceso a mi cuenta mediante el proveedor externo de identidad, con la finalidad de restablecer mis credenciales cuando no pueda iniciar sesión.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuperar acceso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 SP</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuperación de acceso implementada y validada manualmente. SIGET no almacena ni modifica contraseñas locales.</t>
+  </si>
+  <si>
+    <t>E1-H3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito gestionar los roles y permisos de los usuarios, con la finalidad de controlar el acceso de los usuarios a las funcionalidades del sistema.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestión de roles RBAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprovisionamiento y administración de usuarios, roles y permisos mediante API. Permisos derivados de roles locales. Cliente administrativo previsto en PySide6.</t>
+  </si>
+  <si>
+    <t>E2-H4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito registrar un activo tecnológico en el sistema, con la finalidad de mantener un registro actualizado de los equipos tecnológicos disponibles en la empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registrar activo TI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muy Alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro de activos mediante API protegida, con validaciones, control de duplicados y persistencia en las tablas existentes de PostgreSQL. Interfaz administrativa prevista en PySide6.</t>
+  </si>
+  <si>
+    <t>E2-H5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito modificar la información de un activo tecnológico, con la finalidad de mantener actualizados los datos de los equipos registrados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modificar activo TI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modificación de los campos editables mediante API protegida. Conserva el identificador del activo, valida duplicados y registra los cambios en PostgreSQL. Interfaz administrativa prevista en PySide6.</t>
+  </si>
+  <si>
+    <t>E2-H6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito consultar los activos tecnológicos registrados, con la finalidad de conocer la información y estado de los equipos disponibles en la empresa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventario general de activos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consulta de inventario mediante API protegida, con búsqueda y filtros por categoría, ubicación y estado. Interfaz administrativa prevista en PySide6.</t>
+  </si>
+  <si>
+    <t>E3-H7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario solicitante, necesito consultar el catálogo de equipos disponibles y registrar una solicitud de asignación por tipo o categoría de equipo, con la finalidad de disponer del equipamiento necesario para realizar mis actividades.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solicitar asignación de equipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catálogo y formulario Web de solicitud por categoría, con disponibilidad y control de duplicados. El activo físico se selecciona durante la entrega.</t>
+  </si>
+  <si>
+    <t>E3-H8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito gestionar las solicitudes de asignación de equipos, con la finalidad de revisar y controlar las solicitudes realizadas por los usuarios.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprobación de asignaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprobación o rechazo por el Administrador mediante API, con responsable, fecha, motivo de rechazo y auditoría. La aprobación no selecciona ni asigna un activo físico.</t>
+  </si>
+  <si>
+    <t>E3-H9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito consultar las asignaciones de equipos registradas en el sistema, con la finalidad de conocer el estado y la información de las asignaciones realizadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consultar asignaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consulta de asignaciones activas y finalizadas mediante API, con búsqueda por usuario y equipo y filtros por los estados existentes. Interfaz administrativa prevista en PySide6.</t>
+  </si>
+  <si>
+    <t>E3-H20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito registrar la entrega física de un activo compatible con una solicitud de asignación aprobada, con la finalidad de formalizar la asignación y mantener actualizado el estado del activo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registrar entrega de equipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrega de un activo disponible y compatible con una solicitud aprobada. Selección manual, creación de la asignación y actualización transaccional de estados. Lectura de códigos prevista en E8-H19.</t>
+  </si>
+  <si>
+    <t>E4-H10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito registrar la devolución de un equipo asignado, con la finalidad de cerrar la asignación y dejar constancia de la recepción física del activo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registrar devolución de equipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepción y evaluación inicial en una misma operación de API, con cierre de la asignación, fecha y responsable. Interfaz técnica prevista en PySide6.</t>
+  </si>
+  <si>
+    <t>E4-H11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito evaluar y registrar el estado en que se recibe un equipo devuelto, con la finalidad de determinar si puede volver a estar disponible o requiere revisión técnica.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registrar estado de equipo devuelto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipo operativo a Disponible. Con daño o falla, a En revisión, generando o asociando un ticket. Evaluación integrada con la devolución. Diagnóstico y órdenes de trabajo corresponden a historias posteriores.</t>
+  </si>
+  <si>
+    <t>E5-H13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario solicitante, necesito registrar una solicitud de soporte mediante un ticket, con la finalidad de informar un incidente o solicitar un servicio al área de soporte técnico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levantar ticket Service Desk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creación inicial de tickets mediante formulario Web y API, con confirmación, estado inicial, prevención de duplicados y activo opcional autorizado según el rol.</t>
+  </si>
+  <si>
+    <t>E4-H12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito consultar el historial de asignaciones, devoluciones y estados de un equipo, con la finalidad de conocer su uso y situación a lo largo del tiempo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Historial y trazabilidad del equipo</t>
+  </si>
+  <si>
+    <t>Planificada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se registran asignaciones, devoluciones y cambios de estado del activo. Queda pendiente la consulta integrada del historial por equipo y su interfaz administrativa.</t>
+  </si>
+  <si>
+    <t>E5-H14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema o Técnico de soporte, necesito gestionar los tickets de soporte según los permisos de mi rol, con la finalidad de asignar responsables, atender las solicitudes y mantener actualizado su estado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestionar tickets de soporte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Existe consulta y creación inicial de tickets por API. Quedan pendientes la asignación y reasignación de responsables, la atención, los cambios de estado, la resolución y el seguimiento del SLA.</t>
+  </si>
+  <si>
+    <t>E5-H15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario solicitante, necesito consultar el estado de mis tickets de soporte, con la finalidad de conocer el avance y estado de las solicitudes realizadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguimiento de tickets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Existe consulta de tickets propios mediante API. Queda pendiente el portal Web de seguimiento del avance, estado y resolución.</t>
+  </si>
+  <si>
+    <t>E6-H16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito registrar el diagnóstico y gestionar la orden de trabajo asociada a un ticket, con la finalidad de documentar la falla detectada y la intervención técnica requerida sobre el activo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro de diagnósticos y OT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Módulo de taller en PySide6 vinculado a tickets, activos y órdenes de trabajo. La orden de trabajo se abre desde un ticket asociado a un activo en estado ‘En revisión’ e inicia en estado ‘En Diagnóstico’. Al iniciar la intervención técnica, la orden pasa a ‘En Reparación’ y el activo pasa a ‘En reparación’.</t>
+  </si>
+  <si>
+    <t>E10-H23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario solicitante, necesito recibir notificaciones por correo sobre el estado de mis solicitudes, con la finalidad de estar informado oportunamente sobre vencimientos o actualizaciones de servicio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notificaciones por correo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alertas transaccionales mediante una API REST externa de correo ante cambios relevantes. Un fallo de notificación no revierte la operación principal y su tratamiento se realiza conforme a RNF20.</t>
+  </si>
+  <si>
+    <t>E6-H17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito registrar el cierre y resolución de una reparación, con la finalidad de certificar la operatividad del equipo para que vuelva a estar disponible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cierre técnico de reparación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cierra la OT, actualiza el estado operativo del activo y permite completar el proceso técnico.</t>
+  </si>
+  <si>
+    <t>E6-H24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito pausar una orden de trabajo por espera de repuestos o reasignarla a otro Técnico de soporte, con la finalidad de transparentar los cuellos de botella y mantener correctamente registrada la medición del tiempo de resolución (SLA).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pausa o derivación de OT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manejo de pausas, reanudaciones y reasignaciones dentro del ciclo de reparación.</t>
+  </si>
+  <si>
+    <t>E7-H18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito registrar los repuestos utilizados en una reparación, con la finalidad de descontar el stock utilizado y mantener el control de piezas de recambio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asignación de repuestos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Imputación de repuestos a órdenes de trabajo y actualización transaccional de existencias.</t>
+  </si>
+  <si>
+    <t>E7-H25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito registrar el ingreso y compra de nuevos repuestos, con la finalidad de mantener abastecido el inventario de piezas para reparaciones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carga de stock de repuestos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registro de nuevas existencias y actualización del inventario de repuestos.</t>
+  </si>
+  <si>
+    <t>E7-H26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito visualizar alertas automáticas ante repuestos bajo el stock mínimo, con la finalidad de gestionar oportunamente las adquisiciones y evitar quiebres en taller.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerta de stock crítico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de umbrales mínimos y visualización de piezas en estado crítico.</t>
+  </si>
+  <si>
+    <t>E8-H19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Técnico de soporte, necesito leer códigos de barra o QR de los equipos, con la finalidad de identificar con precisión los activos durante su entrega, devolución y operación técnica.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura de códigos QR/Barras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura local mediante lector físico USB HID en PySide6, principalmente durante los procesos de entrega y devolución. Esta lectura no se contabiliza como una API externa, conforme a RNF19.</t>
+  </si>
+  <si>
+    <t>E8-H27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito generar e imprimir etiquetas con código QR para activos nuevos, con la finalidad de rotular físicamente los equipos que ingresan a la flota institucional.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación de códigos QR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación de códigos QR mediante la API externa definida para SIGET, asociándolos al activo correspondiente; impresión y reimpresión de etiquetas desde la aplicación de Escritorio.</t>
+  </si>
+  <si>
+    <t>E9-H21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito consultar reportes de fallas y tiempos de atención, con la finalidad de evaluar el rendimiento del servicio y apoyar la toma de decisiones sobre el parque tecnológico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reportes y métricas de soporte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Métricas de SLA, tiempos de atención y recurrencia de fallas basadas en datos históricos.</t>
+  </si>
+  <si>
+    <t>E9-H22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito consultar el registro histórico de operaciones y eventos críticos, con la finalidad de auditar las acciones realizadas sobre los activos y solicitudes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitácora de auditoría</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se registran operaciones críticas en la bitácora. Quedan pendientes la consulta y el filtrado administrativos, con acceso RBAC y sin modificación ni eliminación, conforme a RNF10 y RNF22.</t>
+  </si>
+  <si>
+    <t>E9-H28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Administrador del sistema, necesito exportar informes ejecutivos del estado y valorización del parque tecnológico, con la finalidad de respaldar auditorías contables e inversiones de TI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reporte consolidado de parque TI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación de informes consolidados y exportación a PDF/Excel.</t>
+  </si>
+  <si>
+    <t>E10-H29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario solicitante, necesito visualizar un centro de notificaciones dentro de la plataforma, con la finalidad de enterarme de avisos urgentes aunque no revise mi correo electrónico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centro de avisos en plataforma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centro de notificaciones internas asociado a eventos de tickets y asignaciones.</t>
+  </si>
+  <si>
+    <t>E5-H30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como un Usuario solicitante, necesito calificar la atención recibida al cerrarse un ticket de soporte, con la finalidad de aportar retroalimentación sobre la calidad del servicio técnico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calificación de servicio (CSAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluación posterior al cierre de tickets y generación de métricas de satisfacción.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pila de Producto (Product Backlog): Instructivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elaborado por: pmoinformatica.com</t>
+  </si>
+  <si>
+    <t>Columna</t>
   </si>
   <si>
     <t>Instrucciones</t>
   </si>
   <si>
-    <t>E1-H1</t>
-  </si>
-  <si>
-    <t>Como un Usuario de SIGET, necesito iniciar sesión en el sistema mediante el proveedor externo de identidad, con la finalidad de acceder a las funcionalidades autorizadas según mi rol.</t>
-  </si>
-  <si>
-    <t>Iniciar sesión</t>
-  </si>
-  <si>
-    <t>Planificada</t>
-  </si>
-  <si>
-    <t>3 SP</t>
-  </si>
-  <si>
-    <t>Sprint 4</t>
-  </si>
-  <si>
-    <t>Código que identifica a la historia de forma unívoca, una vez asignado, no debe ser re-usado en otra historia, ni siquiera si la historia es descartada. El código identifica la historia en otros documentos, como por ejemplo la plantilla de historias de usuario.</t>
-  </si>
-  <si>
-    <t>Alta</t>
-  </si>
-  <si>
-    <t>Autenticación mediante proveedor externo de identidad para los distintos perfiles de SIGET; una vez validada la identidad, el sistema aplica el control de acceso RBAC local conforme a RNF02 y RNF03.</t>
+    <t xml:space="preserve">Código que identifica a la historia de forma unívoca, una vez asignado, no debe ser re-usado en otra historia, ni siquiera si la historia es descartada. El código identifica la historia en otros documentos, como por ejemplo la plantilla de historias de usuario.</t>
   </si>
   <si>
     <t xml:space="preserve">Nombre de la historia, el cual debe ser el mismo que se utiliza en otros documentos. Se puede utilizar el formato siguiente:
@@ -93,52 +471,7 @@
 </t>
   </si>
   <si>
-    <t>E1-H2</t>
-  </si>
-  <si>
-    <t>Como un Usuario de SIGET, necesito recuperar el acceso a mi cuenta mediante el proveedor externo de identidad, con la finalidad de restablecer mis credenciales cuando no pueda iniciar sesión.</t>
-  </si>
-  <si>
-    <t>Recuperar acceso</t>
-  </si>
-  <si>
-    <t>2 SP</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>La recuperación de credenciales es gestionada por el proveedor externo de identidad. SIGET no almacena ni modifica contraseñas locales.</t>
-  </si>
-  <si>
-    <t>Título de la historia alternativo a la descripción, que servirá para identificar más fácilmente la historia sin tener que repetir todo su enunciado. Se puede utilizar por ejemplo el nombre de la funcionalidad o requerimiento que se pretende desarrollar.</t>
-  </si>
-  <si>
-    <t>E1-H3</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito gestionar los roles y permisos de los usuarios, con la finalidad de controlar el acceso de los usuarios a las funcionalidades del sistema.</t>
-  </si>
-  <si>
-    <t>Gestión de roles RBAC</t>
-  </si>
-  <si>
-    <t>5 SP</t>
-  </si>
-  <si>
-    <t>Administración funcional de roles y permisos para Usuario solicitante, Técnico de soporte y Administrador del sistema; control de acceso conforme a RNF02.</t>
-  </si>
-  <si>
-    <t>E2-H4</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito registrar un activo tecnológico en el sistema, con la finalidad de mantener un registro actualizado de los equipos tecnológicos disponibles en la empresa.</t>
-  </si>
-  <si>
-    <t>Registrar activo TI</t>
-  </si>
-  <si>
-    <t>Muy Alta</t>
+    <t xml:space="preserve">Título de la historia alternativo a la descripción, que servirá para identificar más fácilmente la historia sin tener que repetir todo su enunciado. Se puede utilizar por ejemplo el nombre de la funcionalidad o requerimiento que se pretende desarrollar.</t>
   </si>
   <si>
     <t xml:space="preserve">Identifica los posibles estados de la historia durante su ciclo de vida:
@@ -150,378 +483,48 @@
 </t>
   </si>
   <si>
-    <t>Persistencia relacional en módulo de activos en PostgreSQL.</t>
+    <t xml:space="preserve">Medida del esfuerzo (tamaño) que implica desarrollar la historia, existen distintos métodos para medirlo, un ejemplo es los “puntos de historia” una medida de complejidad no necesariamente relacionado con jornadas o días. Otra forma de medirlo es con días o jornadas ideales.</t>
   </si>
   <si>
-    <t>E2-H5</t>
+    <t xml:space="preserve">Iteración o Sprint al que se asigna la historia. Esta asignación puede cambiar en cada iteración donde se haga la revisión de la pila de producto (ProductBacklogReview), según las prioridades indicadas por el dueño de producto. Por medio de este campo se puede crear un “Plan de Salidas a Productivo” (Release Plan).</t>
   </si>
   <si>
-    <t>Como un Administrador del sistema, necesito modificar la información de un activo tecnológico, con la finalidad de mantener actualizados los datos de los equipos registrados.</t>
+    <t xml:space="preserve">Siguiendo el marco de trabajo ágil y Scrum, se le deben asignar prioridades a las historias, según las instrucciones del dueño de producto (ProductOwner). De esta forma pueden ordenarse. Las historias de mayor prioridad deben ser las que agregan más valor al negocio, y deben ser originadas en sus necesidades.</t>
   </si>
   <si>
-    <t>Modificar activo TI</t>
-  </si>
-  <si>
-    <t>Actualización de especificaciones técnicas, números de serie y estado operativo.</t>
-  </si>
-  <si>
-    <t>Medida del esfuerzo (tamaño) que implica desarrollar la historia, existen distintos métodos para medirlo, un ejemplo es los “puntos de historia” una medida de complejidad no necesariamente relacionado con jornadas o días. Otra forma de medirlo es con días o jornadas ideales.</t>
-  </si>
-  <si>
-    <t>E2-H6</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito consultar los activos tecnológicos registrados, con la finalidad de conocer la información y estado de los equipos disponibles en la empresa.</t>
-  </si>
-  <si>
-    <t>Inventario general de activos</t>
-  </si>
-  <si>
-    <t>Vistas administrativas con filtros por categoría, sede y estado operativo.</t>
-  </si>
-  <si>
-    <t>Iteración o Sprint al que se asigna la historia. Esta asignación puede cambiar en cada iteración donde se haga la revisión de la pila de producto (ProductBacklogReview), según las prioridades indicadas por el dueño de producto. Por medio de este campo se puede crear un “Plan de Salidas a Productivo” (Release Plan).</t>
-  </si>
-  <si>
-    <t>E3-H7</t>
-  </si>
-  <si>
-    <t>Como un Usuario solicitante, necesito consultar el catálogo de equipos disponibles y registrar una solicitud de asignación por tipo o categoría de equipo, con la finalidad de disponer del equipamiento necesario para realizar mis actividades.</t>
-  </si>
-  <si>
-    <t>Solicitar asignación de equipo</t>
-  </si>
-  <si>
-    <t>El Portal Web permite consultar el catálogo y la disponibilidad por tipo o categoría. La solicitud registra el tipo o categoría requerida, no un activo físico serializado específico.</t>
-  </si>
-  <si>
-    <t>Siguiendo el marco de trabajo ágil y Scrum, se le deben asignar prioridades a las historias, según las instrucciones del dueño de producto (ProductOwner). De esta forma pueden ordenarse. Las historias de mayor prioridad deben ser las que agregan más valor al negocio, y deben ser originadas en sus necesidades.</t>
-  </si>
-  <si>
-    <t>E3-H8</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito gestionar las solicitudes de asignación de equipos, con la finalidad de revisar y controlar las solicitudes realizadas por los usuarios.</t>
-  </si>
-  <si>
-    <t>Aprobación de asignaciones</t>
-  </si>
-  <si>
-    <t>Sprint 5</t>
-  </si>
-  <si>
-    <t>El Administrador del sistema aprueba o rechaza la solicitud considerando el tipo o categoría requerida y la disponibilidad de inventario. El activo físico específico se selecciona posteriormente durante la entrega.</t>
-  </si>
-  <si>
-    <t>Comentarios o detalles relacionadas que expliquen la historia. Para definiciones de mayor longitud deben usarse documentos externos, por ejemplo la plantilla de historias de usuario.</t>
-  </si>
-  <si>
-    <t>E3-H9</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito consultar las asignaciones de equipos registradas en el sistema, con la finalidad de conocer el estado y la información de las asignaciones realizadas.</t>
-  </si>
-  <si>
-    <t>Consultar asignaciones</t>
-  </si>
-  <si>
-    <t>Seguimiento de asignaciones activas, vencidas y completadas.</t>
-  </si>
-  <si>
-    <t>E3-H20</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito registrar la entrega física de un activo compatible con una solicitud de asignación aprobada, con la finalidad de formalizar la asignación y mantener actualizado el estado del activo.</t>
-  </si>
-  <si>
-    <t>Registrar entrega de equipo</t>
-  </si>
-  <si>
-    <t>Durante la entrega, el Técnico de soporte selecciona e identifica un activo disponible compatible con la solicitud aprobada, registra la asignación, actualiza el activo a estado “Asignado” y marca la solicitud como atendida. Puede utilizar la identificación mediante código de E8-H19.</t>
-  </si>
-  <si>
-    <t>E4-H10</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito registrar la devolución de un equipo asignado, con la finalidad de cerrar la asignación y dejar constancia de la recepción física del activo.</t>
-  </si>
-  <si>
-    <t>Registrar devolución de equipo</t>
-  </si>
-  <si>
-    <t>El Técnico de soporte registra la recepción del activo, fecha y hora de devolución, cierra la asignación activa y continúa con la evaluación del estado del equipo definida en E4-H11.</t>
-  </si>
-  <si>
-    <t>E4-H11</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito evaluar y registrar el estado en que se recibe un equipo devuelto, con la finalidad de determinar si puede volver a estar disponible o requiere revisión técnica.</t>
-  </si>
-  <si>
-    <t>Registrar estado de equipo devuelto</t>
-  </si>
-  <si>
-    <t>Si el equipo se encuentra operativo, pasa a ‘Disponible’. Si presenta una falla, pasa a ‘En revisión’ y se genera o asocia un ticket de soporte para continuar el diagnóstico. Si corresponde abrir una orden de trabajo, esta inicia en estado ‘En Diagnóstico’ mientras el activo permanece ‘En revisión’. El activo pasa a ‘En reparación’ únicamente cuando comienza la intervención técnica de reparación.</t>
-  </si>
-  <si>
-    <t>E5-H13</t>
-  </si>
-  <si>
-    <t>Como un Usuario solicitante, necesito registrar una solicitud de soporte mediante un ticket, con la finalidad de informar un incidente o solicitar un servicio al área de soporte técnico.</t>
-  </si>
-  <si>
-    <t>Levantar ticket Service Desk</t>
-  </si>
-  <si>
-    <t>Portal web para registro de incidentes y requerimientos de soporte.</t>
-  </si>
-  <si>
-    <t>E4-H12</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito consultar el historial de asignaciones, devoluciones y estados de un equipo, con la finalidad de conocer su uso y situación a lo largo del tiempo.</t>
-  </si>
-  <si>
-    <t>Historial y trazabilidad del equipo</t>
-  </si>
-  <si>
-    <t>Sprint 6</t>
-  </si>
-  <si>
-    <t>Consulta histórica vinculada al identificador del activo, asignaciones, devoluciones y usuarios relacionados.</t>
-  </si>
-  <si>
-    <t>E5-H14</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema o Técnico de soporte, necesito gestionar los tickets de soporte según los permisos de mi rol, con la finalidad de asignar responsables, atender las solicitudes y mantener actualizado su estado.</t>
-  </si>
-  <si>
-    <t>Gestionar tickets de soporte</t>
-  </si>
-  <si>
-    <t>El Administrador del sistema asigna o reasigna tickets a Técnicos de soporte. El Técnico gestiona los tickets asignados, actualiza sus estados, registra la atención y resolución y mantiene la trazabilidad del SLA.</t>
-  </si>
-  <si>
-    <t>E5-H15</t>
-  </si>
-  <si>
-    <t>Como un Usuario solicitante, necesito consultar el estado de mis tickets de soporte, con la finalidad de conocer el avance y estado de las solicitudes realizadas.</t>
-  </si>
-  <si>
-    <t>Seguimiento de tickets</t>
-  </si>
-  <si>
-    <t>Portal web para consulta del avance, estado y resolución de tickets.</t>
-  </si>
-  <si>
-    <t>E6-H16</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito registrar el diagnóstico y gestionar la orden de trabajo asociada a un ticket, con la finalidad de documentar la falla detectada y la intervención técnica requerida sobre el activo.</t>
-  </si>
-  <si>
-    <t>Registro de diagnósticos y OT</t>
-  </si>
-  <si>
-    <t>8 SP</t>
-  </si>
-  <si>
-    <t>Módulo de taller en PySide6 vinculado a tickets, activos y órdenes de trabajo. La orden de trabajo se abre desde un ticket asociado a un activo en estado ‘En revisión’ e inicia en estado ‘En Diagnóstico’. Al iniciar la intervención técnica, la orden pasa a ‘En Reparación’ y el activo pasa a ‘En reparación’.</t>
-  </si>
-  <si>
-    <t>E10-H23</t>
-  </si>
-  <si>
-    <t>Como un Usuario solicitante, necesito recibir notificaciones por correo sobre el estado de mis solicitudes, con la finalidad de estar informado oportunamente sobre vencimientos o actualizaciones de servicio.</t>
-  </si>
-  <si>
-    <t>Notificaciones por correo</t>
-  </si>
-  <si>
-    <t>Alertas transaccionales mediante una API REST externa de correo ante cambios relevantes. Un fallo de notificación no revierte la operación principal y su tratamiento se realiza conforme a RNF20.</t>
-  </si>
-  <si>
-    <t>E6-H17</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito registrar el cierre y resolución de una reparación, con la finalidad de certificar la operatividad del equipo para que vuelva a estar disponible.</t>
-  </si>
-  <si>
-    <t>Cierre técnico de reparación</t>
-  </si>
-  <si>
-    <t>Sprint 7</t>
-  </si>
-  <si>
-    <t>Cierra la OT, actualiza el estado operativo del activo y permite completar el proceso técnico.</t>
-  </si>
-  <si>
-    <t>E6-H24</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito pausar una orden de trabajo por espera de repuestos o reasignarla a otro Técnico de soporte, con la finalidad de transparentar los cuellos de botella y mantener correctamente registrada la medición del tiempo de resolución (SLA).</t>
-  </si>
-  <si>
-    <t>Pausa o derivación de OT</t>
-  </si>
-  <si>
-    <t>Manejo de pausas, reanudaciones y reasignaciones dentro del ciclo de reparación.</t>
-  </si>
-  <si>
-    <t>E7-H18</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito registrar los repuestos utilizados en una reparación, con la finalidad de descontar el stock utilizado y mantener el control de piezas de recambio.</t>
-  </si>
-  <si>
-    <t>Asignación de repuestos</t>
-  </si>
-  <si>
-    <t>Imputación de repuestos a órdenes de trabajo y actualización transaccional de existencias.</t>
-  </si>
-  <si>
-    <t>E7-H25</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito registrar el ingreso y compra de nuevos repuestos, con la finalidad de mantener abastecido el inventario de piezas para reparaciones.</t>
-  </si>
-  <si>
-    <t>Carga de stock de repuestos</t>
-  </si>
-  <si>
-    <t>Registro de nuevas existencias y actualización del inventario de repuestos.</t>
-  </si>
-  <si>
-    <t>E7-H26</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito visualizar alertas automáticas ante repuestos bajo el stock mínimo, con la finalidad de gestionar oportunamente las adquisiciones y evitar quiebres en taller.</t>
-  </si>
-  <si>
-    <t>Alerta de stock crítico</t>
-  </si>
-  <si>
-    <t>Control de umbrales mínimos y visualización de piezas en estado crítico.</t>
-  </si>
-  <si>
-    <t>E8-H19</t>
-  </si>
-  <si>
-    <t>Como un Técnico de soporte, necesito leer códigos de barra o QR de los equipos, con la finalidad de identificar con precisión los activos durante su entrega, devolución y operación técnica.</t>
-  </si>
-  <si>
-    <t>Lectura de códigos QR/Barras</t>
-  </si>
-  <si>
-    <t>Lectura local mediante lector físico USB HID en PySide6, principalmente durante los procesos de entrega y devolución. Esta lectura no se contabiliza como una API externa, conforme a RNF19.</t>
-  </si>
-  <si>
-    <t>E8-H27</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito generar e imprimir etiquetas con código QR para activos nuevos, con la finalidad de rotular físicamente los equipos que ingresan a la flota institucional.</t>
-  </si>
-  <si>
-    <t>Generación de códigos QR</t>
-  </si>
-  <si>
-    <t>Sprint 8</t>
-  </si>
-  <si>
-    <t>Generación de códigos QR mediante la API externa definida para SIGET, asociándolos al activo correspondiente; impresión y reimpresión de etiquetas desde la aplicación de Escritorio.</t>
-  </si>
-  <si>
-    <t>E9-H21</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito consultar reportes de fallas y tiempos de atención, con la finalidad de evaluar el rendimiento del servicio y apoyar la toma de decisiones sobre el parque tecnológico.</t>
-  </si>
-  <si>
-    <t>Reportes y métricas de soporte</t>
-  </si>
-  <si>
-    <t>Métricas de SLA, tiempos de atención y recurrencia de fallas basadas en datos históricos.</t>
-  </si>
-  <si>
-    <t>E9-H22</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito consultar el registro histórico de operaciones y eventos críticos, con la finalidad de auditar las acciones realizadas sobre los activos y solicitudes.</t>
-  </si>
-  <si>
-    <t>Bitácora de auditoría</t>
-  </si>
-  <si>
-    <t>Consulta y filtrado del registro histórico de operaciones críticas, con acceso restringido mediante RBAC y sin funciones de modificación o eliminación desde la aplicación, conforme a RNF10 y RNF22.</t>
-  </si>
-  <si>
-    <t>E9-H28</t>
-  </si>
-  <si>
-    <t>Como un Administrador del sistema, necesito exportar informes ejecutivos del estado y valorización del parque tecnológico, con la finalidad de respaldar auditorías contables e inversiones de TI.</t>
-  </si>
-  <si>
-    <t>Reporte consolidado de parque TI</t>
-  </si>
-  <si>
-    <t>Generación de informes consolidados y exportación a PDF/Excel.</t>
-  </si>
-  <si>
-    <t>E10-H29</t>
-  </si>
-  <si>
-    <t>Como un Usuario solicitante, necesito visualizar un centro de notificaciones dentro de la plataforma, con la finalidad de enterarme de avisos urgentes aunque no revise mi correo electrónico.</t>
-  </si>
-  <si>
-    <t>Centro de avisos en plataforma</t>
-  </si>
-  <si>
-    <t>Centro de notificaciones internas asociado a eventos de tickets y asignaciones.</t>
-  </si>
-  <si>
-    <t>E5-H30</t>
-  </si>
-  <si>
-    <t>Como un Usuario solicitante, necesito calificar la atención recibida al cerrarse un ticket de soporte, con la finalidad de aportar retroalimentación sobre la calidad del servicio técnico.</t>
-  </si>
-  <si>
-    <t>Calificación de servicio (CSAT)</t>
-  </si>
-  <si>
-    <t>Evaluación posterior al cierre de tickets y generación de métricas de satisfacción.</t>
+    <t xml:space="preserve">Comentarios o detalles relacionadas que expliquen la historia. Para definiciones de mayor longitud deben usarse documentos externos, por ejemplo la plantilla de historias de usuario.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6">
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="28.0"/>
+      <sz val="28.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
+      <sz val="16.000000"/>
       <color rgb="FF1F497D"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="0"/>
       <name val="Calibri"/>
     </font>
@@ -536,7 +539,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -551,88 +554,358 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
-    <border/>
+  <borders count="2">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
-    </border>
-    <border>
-      <left/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <bottom/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+  <cellXfs count="11">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="3" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf fontId="4" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="5" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="4" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -689,7 +962,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -715,7 +988,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -792,7 +1065,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -822,29 +1095,31 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="1.43"/>
+    <col customWidth="1" min="1" max="1" width="1.4299999999999999"/>
     <col customWidth="1" min="2" max="2" width="16.43"/>
-    <col customWidth="1" min="3" max="3" width="57.71"/>
+    <col customWidth="1" min="3" max="3" width="57.710000000000001"/>
     <col customWidth="1" min="4" max="4" width="32.57"/>
-    <col customWidth="1" min="5" max="5" width="13.0"/>
-    <col customWidth="1" min="6" max="6" width="11.86"/>
-    <col customWidth="1" min="7" max="7" width="16.14"/>
-    <col customWidth="1" min="8" max="8" width="17.86"/>
-    <col customWidth="1" min="9" max="9" width="40.29"/>
-    <col customWidth="1" min="10" max="26" width="10.71"/>
+    <col customWidth="1" min="5" max="5" width="13"/>
+    <col customWidth="1" min="6" max="6" width="11.859999999999999"/>
+    <col customWidth="1" min="7" max="7" width="16.140000000000001"/>
+    <col customWidth="1" min="8" max="8" width="17.859999999999999"/>
+    <col customWidth="1" min="9" max="9" width="40.289999999999999"/>
+    <col customWidth="1" min="10" max="26" width="10.710000000000001"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="36">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -874,10 +1149,10 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2">
+    <row r="2" ht="21">
       <c r="A2" s="1"/>
       <c r="B2" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -932,31 +1207,31 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4">
+    <row r="4" ht="28.5">
       <c r="A4" s="1"/>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="I4" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -976,1336 +1251,1336 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" ht="72.0" customHeight="1">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8" t="s">
+    <row r="5" s="5" customFormat="1" ht="42.75">
+      <c r="A5" s="6"/>
+      <c r="B5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="H5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="I5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6"/>
+      <c r="Z5" s="6"/>
+    </row>
+    <row r="6" s="5" customFormat="1" ht="57">
+      <c r="A6" s="6"/>
+      <c r="B6" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="D6" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="G6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="10"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="1"/>
-      <c r="U5" s="1"/>
-      <c r="V5" s="1"/>
-      <c r="W5" s="1"/>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="1"/>
-      <c r="Z5" s="1"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8" t="s">
+      <c r="I6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6"/>
+      <c r="Z6" s="6"/>
+    </row>
+    <row r="7" s="5" customFormat="1" ht="57">
+      <c r="A7" s="6"/>
+      <c r="B7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>17</v>
+      <c r="E7" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="H7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="10"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="1"/>
-      <c r="U6" s="1"/>
-      <c r="V6" s="1"/>
-      <c r="W6" s="1"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="1"/>
-      <c r="Z6" s="1"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8" t="s">
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
+    </row>
+    <row r="8" s="5" customFormat="1" ht="71.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="8" t="s">
+      <c r="I8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="8" t="s">
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
+      <c r="X8" s="6"/>
+      <c r="Y8" s="6"/>
+      <c r="Z8" s="6"/>
+    </row>
+    <row r="9" s="5" customFormat="1" ht="71.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="J7" s="10"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="1"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="1"/>
-      <c r="U7" s="1"/>
-      <c r="V7" s="1"/>
-      <c r="W7" s="1"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="1"/>
-      <c r="Z7" s="1"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="8" t="s">
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
+      <c r="V9" s="6"/>
+      <c r="W9" s="6"/>
+      <c r="X9" s="6"/>
+      <c r="Y9" s="6"/>
+      <c r="Z9" s="6"/>
+    </row>
+    <row r="10" s="5" customFormat="1" ht="57">
+      <c r="A10" s="6"/>
+      <c r="B10" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="C10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="10"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="1"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="1"/>
-      <c r="W8" s="1"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="1"/>
-      <c r="Z8" s="1"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8" t="s">
+      <c r="E10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="6"/>
+      <c r="W10" s="6"/>
+      <c r="X10" s="6"/>
+      <c r="Y10" s="6"/>
+      <c r="Z10" s="6"/>
+    </row>
+    <row r="11" s="5" customFormat="1" ht="57">
+      <c r="A11" s="6"/>
+      <c r="B11" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="8" t="s">
-        <v>17</v>
+      <c r="D11" s="7" t="s">
+        <v>45</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>18</v>
+      <c r="E11" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>19</v>
+      <c r="F11" s="7" t="s">
+        <v>27</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>45</v>
+      <c r="H11" s="7" t="s">
+        <v>33</v>
       </c>
-      <c r="J9" s="10"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="1"/>
-      <c r="U9" s="1"/>
-      <c r="V9" s="1"/>
-      <c r="W9" s="1"/>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="1"/>
-      <c r="Z9" s="1"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8" t="s">
+      <c r="I11" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="6"/>
+      <c r="W11" s="6"/>
+      <c r="X11" s="6"/>
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6"/>
+    </row>
+    <row r="12" s="5" customFormat="1" ht="57">
+      <c r="A12" s="6"/>
+      <c r="B12" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="8" t="s">
-        <v>17</v>
+      <c r="E12" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>18</v>
+      <c r="F12" s="7" t="s">
+        <v>27</v>
       </c>
-      <c r="G10" s="8" t="s">
-        <v>19</v>
+      <c r="G12" s="7" t="s">
+        <v>28</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>21</v>
+      <c r="H12" s="7" t="s">
+        <v>16</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I12" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="J10" s="10"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
-      <c r="S10" s="1"/>
-      <c r="T10" s="1"/>
-      <c r="U10" s="1"/>
-      <c r="V10" s="1"/>
-      <c r="W10" s="1"/>
-      <c r="X10" s="1"/>
-      <c r="Y10" s="1"/>
-      <c r="Z10" s="1"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8" t="s">
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="6"/>
+      <c r="W12" s="6"/>
+      <c r="X12" s="6"/>
+      <c r="Y12" s="6"/>
+      <c r="Z12" s="6"/>
+    </row>
+    <row r="13" s="5" customFormat="1" ht="57">
+      <c r="A13" s="6"/>
+      <c r="B13" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="E13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="I11" s="8" t="s">
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
+    </row>
+    <row r="14" s="5" customFormat="1" ht="71.25">
+      <c r="A14" s="6"/>
+      <c r="B14" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="10"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
-      <c r="S11" s="1"/>
-      <c r="T11" s="1"/>
-      <c r="U11" s="1"/>
-      <c r="V11" s="1"/>
-      <c r="W11" s="1"/>
-      <c r="X11" s="1"/>
-      <c r="Y11" s="1"/>
-      <c r="Z11" s="1"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="7"/>
-      <c r="B12" s="8" t="s">
+      <c r="C14" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="E14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I14" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="6"/>
+      <c r="W14" s="6"/>
+      <c r="X14" s="6"/>
+      <c r="Y14" s="6"/>
+      <c r="Z14" s="6"/>
+    </row>
+    <row r="15" s="5" customFormat="1" ht="57">
+      <c r="A15" s="6"/>
+      <c r="B15" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G12" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="H12" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J12" s="10"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
-      <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="1"/>
-      <c r="U12" s="1"/>
-      <c r="V12" s="1"/>
-      <c r="W12" s="1"/>
-      <c r="X12" s="1"/>
-      <c r="Y12" s="1"/>
-      <c r="Z12" s="1"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7"/>
-      <c r="B13" s="8" t="s">
+      <c r="E15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="6"/>
+      <c r="W15" s="6"/>
+      <c r="X15" s="6"/>
+      <c r="Y15" s="6"/>
+      <c r="Z15" s="6"/>
+    </row>
+    <row r="16" s="5" customFormat="1" ht="71.25">
+      <c r="A16" s="6"/>
+      <c r="B16" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D16" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>17</v>
+      <c r="E16" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>18</v>
+      <c r="F16" s="7" t="s">
+        <v>14</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H13" s="8" t="s">
+      <c r="G16" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="H16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="J13" s="10"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="1"/>
-      <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
-      <c r="V13" s="1"/>
-      <c r="W13" s="1"/>
-      <c r="X13" s="1"/>
-      <c r="Y13" s="1"/>
-      <c r="Z13" s="1"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7"/>
-      <c r="B14" s="8" t="s">
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="6"/>
+      <c r="S16" s="6"/>
+      <c r="T16" s="6"/>
+      <c r="U16" s="6"/>
+      <c r="V16" s="6"/>
+      <c r="W16" s="6"/>
+      <c r="X16" s="6"/>
+      <c r="Y16" s="6"/>
+      <c r="Z16" s="6"/>
+    </row>
+    <row r="17" s="5" customFormat="1" ht="57">
+      <c r="A17" s="6"/>
+      <c r="B17" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D17" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E14" s="8" t="s">
-        <v>17</v>
+      <c r="E17" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>34</v>
+      <c r="F17" s="7" t="s">
+        <v>27</v>
       </c>
-      <c r="G14" s="8" t="s">
-        <v>60</v>
+      <c r="G17" s="7" t="s">
+        <v>28</v>
       </c>
-      <c r="H14" s="8" t="s">
-        <v>39</v>
+      <c r="H17" s="7" t="s">
+        <v>33</v>
       </c>
-      <c r="I14" s="8" t="s">
+      <c r="I17" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="J14" s="10"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
-      <c r="S14" s="1"/>
-      <c r="T14" s="1"/>
-      <c r="U14" s="1"/>
-      <c r="V14" s="1"/>
-      <c r="W14" s="1"/>
-      <c r="X14" s="1"/>
-      <c r="Y14" s="1"/>
-      <c r="Z14" s="1"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7"/>
-      <c r="B15" s="8" t="s">
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6"/>
+      <c r="T17" s="6"/>
+      <c r="U17" s="6"/>
+      <c r="V17" s="6"/>
+      <c r="W17" s="6"/>
+      <c r="X17" s="6"/>
+      <c r="Y17" s="6"/>
+      <c r="Z17" s="6"/>
+    </row>
+    <row r="18" s="5" customFormat="1" ht="57">
+      <c r="A18" s="6"/>
+      <c r="B18" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="E15" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="I15" s="8" t="s">
+      <c r="E18" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="J15" s="10"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="1"/>
-      <c r="U15" s="1"/>
-      <c r="V15" s="1"/>
-      <c r="W15" s="1"/>
-      <c r="X15" s="1"/>
-      <c r="Y15" s="1"/>
-      <c r="Z15" s="1"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8" t="s">
+      <c r="F18" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="H18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="6"/>
+      <c r="S18" s="6"/>
+      <c r="T18" s="6"/>
+      <c r="U18" s="6"/>
+      <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
+      <c r="X18" s="6"/>
+      <c r="Y18" s="6"/>
+      <c r="Z18" s="6"/>
+    </row>
+    <row r="19" s="5" customFormat="1" ht="71.25">
+      <c r="A19" s="6"/>
+      <c r="B19" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I16" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="J16" s="10"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="1"/>
-      <c r="U16" s="1"/>
-      <c r="V16" s="1"/>
-      <c r="W16" s="1"/>
-      <c r="X16" s="1"/>
-      <c r="Y16" s="1"/>
-      <c r="Z16" s="1"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8" t="s">
+      <c r="D19" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="E19" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="6"/>
+      <c r="S19" s="6"/>
+      <c r="T19" s="6"/>
+      <c r="U19" s="6"/>
+      <c r="V19" s="6"/>
+      <c r="W19" s="6"/>
+      <c r="X19" s="6"/>
+      <c r="Y19" s="6"/>
+      <c r="Z19" s="6"/>
+    </row>
+    <row r="20" s="5" customFormat="1" ht="42.75">
+      <c r="A20" s="6"/>
+      <c r="B20" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="E17" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="I17" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="J17" s="10"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="1"/>
-      <c r="U17" s="1"/>
-      <c r="V17" s="1"/>
-      <c r="W17" s="1"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="1"/>
-      <c r="Z17" s="1"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="E20" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="6"/>
+      <c r="S20" s="6"/>
+      <c r="T20" s="6"/>
+      <c r="U20" s="6"/>
+      <c r="V20" s="6"/>
+      <c r="W20" s="6"/>
+      <c r="X20" s="6"/>
+      <c r="Y20" s="6"/>
+      <c r="Z20" s="6"/>
+    </row>
+    <row r="21" s="5" customFormat="1" ht="99.75">
+      <c r="A21" s="6"/>
+      <c r="B21" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G18" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="H18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="8" t="s">
+      <c r="D21" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J18" s="10"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="1"/>
-      <c r="U18" s="1"/>
-      <c r="V18" s="1"/>
-      <c r="W18" s="1"/>
-      <c r="X18" s="1"/>
-      <c r="Y18" s="1"/>
-      <c r="Z18" s="1"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8" t="s">
+      <c r="E21" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="G21" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
+      <c r="V21" s="6"/>
+      <c r="W21" s="6"/>
+      <c r="X21" s="6"/>
+      <c r="Y21" s="6"/>
+      <c r="Z21" s="6"/>
+    </row>
+    <row r="22" s="5" customFormat="1" ht="71.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I19" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="J19" s="10"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="1"/>
-      <c r="U19" s="1"/>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7"/>
-      <c r="B20" s="8" t="s">
+      <c r="D22" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="E22" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="6"/>
+      <c r="T22" s="6"/>
+      <c r="U22" s="6"/>
+      <c r="V22" s="6"/>
+      <c r="W22" s="6"/>
+      <c r="X22" s="6"/>
+      <c r="Y22" s="6"/>
+      <c r="Z22" s="6"/>
+    </row>
+    <row r="23" s="5" customFormat="1" ht="42.75">
+      <c r="A23" s="6"/>
+      <c r="B23" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E20" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I20" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="J20" s="10"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="1"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="1"/>
-      <c r="U20" s="1"/>
-      <c r="V20" s="1"/>
-      <c r="W20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="1"/>
-      <c r="Z20" s="1"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="7"/>
-      <c r="B21" s="8" t="s">
+      <c r="D23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="E23" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="H23" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E21" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="8" t="s">
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="6"/>
+      <c r="S23" s="6"/>
+      <c r="T23" s="6"/>
+      <c r="U23" s="6"/>
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
+      <c r="Z23" s="6"/>
+    </row>
+    <row r="24" s="5" customFormat="1" ht="71.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="G21" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="I21" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="J21" s="10"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="1"/>
-      <c r="U21" s="1"/>
-      <c r="V21" s="1"/>
-      <c r="W21" s="1"/>
-      <c r="X21" s="1"/>
-      <c r="Y21" s="1"/>
-      <c r="Z21" s="1"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="7"/>
-      <c r="B22" s="8" t="s">
+      <c r="D24" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="E24" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="J24" s="6"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="6"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="6"/>
+      <c r="S24" s="6"/>
+      <c r="T24" s="6"/>
+      <c r="U24" s="6"/>
+      <c r="V24" s="6"/>
+      <c r="W24" s="6"/>
+      <c r="X24" s="6"/>
+      <c r="Y24" s="6"/>
+      <c r="Z24" s="6"/>
+    </row>
+    <row r="25" s="5" customFormat="1" ht="42.75">
+      <c r="A25" s="6"/>
+      <c r="B25" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E22" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I22" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="10"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
-      <c r="P22" s="1"/>
-      <c r="Q22" s="1"/>
-      <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="1"/>
-      <c r="U22" s="1"/>
-      <c r="V22" s="1"/>
-      <c r="W22" s="1"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="1"/>
-      <c r="Z22" s="1"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="7"/>
-      <c r="B23" s="8" t="s">
+      <c r="D25" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="E25" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="8" t="s">
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="6"/>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+      <c r="V25" s="6"/>
+      <c r="W25" s="6"/>
+      <c r="X25" s="6"/>
+      <c r="Y25" s="6"/>
+      <c r="Z25" s="6"/>
+    </row>
+    <row r="26" s="5" customFormat="1" ht="42.75">
+      <c r="A26" s="6"/>
+      <c r="B26" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="E23" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G23" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H23" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I23" s="8" t="s">
+      <c r="D26" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="J23" s="10"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
-      <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="1"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="1"/>
-      <c r="W23" s="1"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="1"/>
-      <c r="Z23" s="1"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="7"/>
-      <c r="B24" s="8" t="s">
+      <c r="E26" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I26" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
+      <c r="U26" s="6"/>
+      <c r="V26" s="6"/>
+      <c r="W26" s="6"/>
+      <c r="X26" s="6"/>
+      <c r="Y26" s="6"/>
+      <c r="Z26" s="6"/>
+    </row>
+    <row r="27" s="5" customFormat="1" ht="57">
+      <c r="A27" s="6"/>
+      <c r="B27" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="E24" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I24" s="8" t="s">
+      <c r="D27" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="J24" s="10"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
-      <c r="N24" s="1"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="1"/>
-      <c r="U24" s="1"/>
-      <c r="V24" s="1"/>
-      <c r="W24" s="1"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="1"/>
-      <c r="Z24" s="1"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="7"/>
-      <c r="B25" s="8" t="s">
+      <c r="E27" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+      <c r="R27" s="6"/>
+      <c r="S27" s="6"/>
+      <c r="T27" s="6"/>
+      <c r="U27" s="6"/>
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
+      <c r="X27" s="6"/>
+      <c r="Y27" s="6"/>
+      <c r="Z27" s="6"/>
+    </row>
+    <row r="28" s="5" customFormat="1" ht="71.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="E25" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I25" s="8" t="s">
+      <c r="D28" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="J25" s="10"/>
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="1"/>
-      <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="7"/>
-      <c r="B26" s="8" t="s">
+      <c r="E28" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+      <c r="U28" s="6"/>
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
+      <c r="X28" s="6"/>
+      <c r="Y28" s="6"/>
+      <c r="Z28" s="6"/>
+    </row>
+    <row r="29" s="5" customFormat="1" ht="71.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="E26" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H26" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I26" s="8" t="s">
+      <c r="D29" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="J26" s="10"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-      <c r="M26" s="1"/>
-      <c r="N26" s="1"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1"/>
-      <c r="R26" s="1"/>
-      <c r="S26" s="1"/>
-      <c r="T26" s="1"/>
-      <c r="U26" s="1"/>
-      <c r="V26" s="1"/>
-      <c r="W26" s="1"/>
-      <c r="X26" s="1"/>
-      <c r="Y26" s="1"/>
-      <c r="Z26" s="1"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="7"/>
-      <c r="B27" s="8" t="s">
+      <c r="E29" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G29" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="H29" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+      <c r="R29" s="6"/>
+      <c r="S29" s="6"/>
+      <c r="T29" s="6"/>
+      <c r="U29" s="6"/>
+      <c r="V29" s="6"/>
+      <c r="W29" s="6"/>
+      <c r="X29" s="6"/>
+      <c r="Y29" s="6"/>
+      <c r="Z29" s="6"/>
+    </row>
+    <row r="30" s="5" customFormat="1" ht="57">
+      <c r="A30" s="6"/>
+      <c r="B30" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="E27" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I27" s="8" t="s">
+      <c r="C30" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="J27" s="10"/>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="1"/>
-      <c r="N27" s="1"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="1"/>
-      <c r="R27" s="1"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="1"/>
-      <c r="U27" s="1"/>
-      <c r="V27" s="1"/>
-      <c r="W27" s="1"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="1"/>
-      <c r="Z27" s="1"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="7"/>
-      <c r="B28" s="8" t="s">
+      <c r="D30" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="E30" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="D28" s="8" t="s">
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6"/>
+      <c r="M30" s="6"/>
+      <c r="N30" s="6"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="6"/>
+      <c r="R30" s="6"/>
+      <c r="S30" s="6"/>
+      <c r="T30" s="6"/>
+      <c r="U30" s="6"/>
+      <c r="V30" s="6"/>
+      <c r="W30" s="6"/>
+      <c r="X30" s="6"/>
+      <c r="Y30" s="6"/>
+      <c r="Z30" s="6"/>
+    </row>
+    <row r="31" s="5" customFormat="1" ht="71.25">
+      <c r="A31" s="6"/>
+      <c r="B31" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="E28" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G28" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I28" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="J28" s="10"/>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-      <c r="M28" s="1"/>
-      <c r="N28" s="1"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="1"/>
-      <c r="R28" s="1"/>
-      <c r="S28" s="1"/>
-      <c r="T28" s="1"/>
-      <c r="U28" s="1"/>
-      <c r="V28" s="1"/>
-      <c r="W28" s="1"/>
-      <c r="X28" s="1"/>
-      <c r="Y28" s="1"/>
-      <c r="Z28" s="1"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="7"/>
-      <c r="B29" s="8" t="s">
+      <c r="D31" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="E31" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
+      <c r="V31" s="6"/>
+      <c r="W31" s="6"/>
+      <c r="X31" s="6"/>
+      <c r="Y31" s="6"/>
+      <c r="Z31" s="6"/>
+    </row>
+    <row r="32" s="5" customFormat="1" ht="42.75">
+      <c r="A32" s="6"/>
+      <c r="B32" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="E29" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G29" s="8" t="s">
+      <c r="C32" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="H29" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I29" s="8" t="s">
+      <c r="D32" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="J29" s="10"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-      <c r="M29" s="1"/>
-      <c r="N29" s="1"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
-      <c r="U29" s="1"/>
-      <c r="V29" s="1"/>
-      <c r="W29" s="1"/>
-      <c r="X29" s="1"/>
-      <c r="Y29" s="1"/>
-      <c r="Z29" s="1"/>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="7"/>
-      <c r="B30" s="8" t="s">
+      <c r="E32" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
+      <c r="M32" s="6"/>
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6"/>
+      <c r="R32" s="6"/>
+      <c r="S32" s="6"/>
+      <c r="T32" s="6"/>
+      <c r="U32" s="6"/>
+      <c r="V32" s="6"/>
+      <c r="W32" s="6"/>
+      <c r="X32" s="6"/>
+      <c r="Y32" s="6"/>
+      <c r="Z32" s="6"/>
+    </row>
+    <row r="33" s="5" customFormat="1" ht="57">
+      <c r="A33" s="6"/>
+      <c r="B33" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D30" s="8" t="s">
+      <c r="C33" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="E30" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="G30" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="H30" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I30" s="8" t="s">
+      <c r="D33" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="J30" s="10"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
-      <c r="U30" s="1"/>
-      <c r="V30" s="1"/>
-      <c r="W30" s="1"/>
-      <c r="X30" s="1"/>
-      <c r="Y30" s="1"/>
-      <c r="Z30" s="1"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="7"/>
-      <c r="B31" s="8" t="s">
+      <c r="E33" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
+      <c r="R33" s="6"/>
+      <c r="S33" s="6"/>
+      <c r="T33" s="6"/>
+      <c r="U33" s="6"/>
+      <c r="V33" s="6"/>
+      <c r="W33" s="6"/>
+      <c r="X33" s="6"/>
+      <c r="Y33" s="6"/>
+      <c r="Z33" s="6"/>
+    </row>
+    <row r="34" s="5" customFormat="1" ht="42.75">
+      <c r="A34" s="6"/>
+      <c r="B34" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D31" s="8" t="s">
+      <c r="C34" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="E31" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="H31" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I31" s="8" t="s">
+      <c r="D34" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="J31" s="10"/>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
-      <c r="S31" s="1"/>
-      <c r="T31" s="1"/>
-      <c r="U31" s="1"/>
-      <c r="V31" s="1"/>
-      <c r="W31" s="1"/>
-      <c r="X31" s="1"/>
-      <c r="Y31" s="1"/>
-      <c r="Z31" s="1"/>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="7"/>
-      <c r="B32" s="8" t="s">
+      <c r="E34" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C32" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I32" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="J32" s="10"/>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
-      <c r="M32" s="1"/>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="1"/>
-      <c r="R32" s="1"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="1"/>
-      <c r="U32" s="1"/>
-      <c r="V32" s="1"/>
-      <c r="W32" s="1"/>
-      <c r="X32" s="1"/>
-      <c r="Y32" s="1"/>
-      <c r="Z32" s="1"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="7"/>
-      <c r="B33" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F33" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="J33" s="10"/>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
-      <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
-      <c r="Q33" s="1"/>
-      <c r="R33" s="1"/>
-      <c r="S33" s="1"/>
-      <c r="T33" s="1"/>
-      <c r="U33" s="1"/>
-      <c r="V33" s="1"/>
-      <c r="W33" s="1"/>
-      <c r="X33" s="1"/>
-      <c r="Y33" s="1"/>
-      <c r="Z33" s="1"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="7"/>
-      <c r="B34" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="H34" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="I34" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="J34" s="10"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="1"/>
-      <c r="R34" s="1"/>
-      <c r="S34" s="1"/>
-      <c r="T34" s="1"/>
-      <c r="U34" s="1"/>
-      <c r="V34" s="1"/>
-      <c r="W34" s="1"/>
-      <c r="X34" s="1"/>
-      <c r="Y34" s="1"/>
-      <c r="Z34" s="1"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
+      <c r="L34" s="6"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6"/>
+      <c r="R34" s="6"/>
+      <c r="S34" s="6"/>
+      <c r="T34" s="6"/>
+      <c r="U34" s="6"/>
+      <c r="V34" s="6"/>
+      <c r="W34" s="6"/>
+      <c r="X34" s="6"/>
+      <c r="Y34" s="6"/>
+      <c r="Z34" s="6"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="1"/>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
@@ -29345,32 +29620,33 @@
       <c r="Z1000" s="1"/>
     </row>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.7480314960629921" footer="0.0" header="0.0" left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921"/>
-  <pageSetup scale="70" orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.74803149606299213" bottom="0.74803149606299213" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="70" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="1.57"/>
-    <col customWidth="1" min="2" max="2" width="27.71"/>
-    <col customWidth="1" min="3" max="3" width="86.0"/>
-    <col customWidth="1" min="4" max="4" width="2.86"/>
+    <col customWidth="1" min="1" max="1" width="1.5700000000000001"/>
+    <col customWidth="1" min="2" max="2" width="27.710000000000001"/>
+    <col customWidth="1" min="3" max="3" width="86"/>
+    <col customWidth="1" min="4" max="4" width="2.8599999999999999"/>
     <col customWidth="1" min="5" max="6" width="11.43"/>
-    <col customWidth="1" min="7" max="26" width="10.71"/>
+    <col customWidth="1" min="7" max="26" width="10.710000000000001"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>144</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -29399,8 +29675,8 @@
     </row>
     <row r="2">
       <c r="A2" s="1"/>
-      <c r="B2" s="4" t="s">
-        <v>3</v>
+      <c r="B2" s="8" t="s">
+        <v>145</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -29457,11 +29733,11 @@
     </row>
     <row r="4">
       <c r="A4" s="1"/>
-      <c r="B4" s="6" t="s">
-        <v>11</v>
+      <c r="B4" s="9" t="s">
+        <v>146</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>13</v>
+      <c r="C4" s="9" t="s">
+        <v>147</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -29489,11 +29765,11 @@
     </row>
     <row r="5">
       <c r="A5" s="1"/>
-      <c r="B5" s="9" t="s">
-        <v>4</v>
+      <c r="B5" s="10" t="s">
+        <v>2</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>20</v>
+      <c r="C5" s="10" t="s">
+        <v>148</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -29521,11 +29797,11 @@
     </row>
     <row r="6">
       <c r="A6" s="1"/>
-      <c r="B6" s="9" t="s">
-        <v>5</v>
+      <c r="B6" s="10" t="s">
+        <v>3</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>23</v>
+      <c r="C6" s="10" t="s">
+        <v>149</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -29553,11 +29829,11 @@
     </row>
     <row r="7">
       <c r="A7" s="1"/>
-      <c r="B7" s="9" t="s">
-        <v>6</v>
+      <c r="B7" s="10" t="s">
+        <v>4</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>30</v>
+      <c r="C7" s="10" t="s">
+        <v>150</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -29585,11 +29861,11 @@
     </row>
     <row r="8">
       <c r="A8" s="1"/>
-      <c r="B8" s="9" t="s">
-        <v>7</v>
+      <c r="B8" s="10" t="s">
+        <v>5</v>
       </c>
-      <c r="C8" s="9" t="s">
-        <v>40</v>
+      <c r="C8" s="10" t="s">
+        <v>151</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -29617,11 +29893,11 @@
     </row>
     <row r="9" ht="50.25" customHeight="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="9" t="s">
-        <v>8</v>
+      <c r="B9" s="10" t="s">
+        <v>6</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>46</v>
+      <c r="C9" s="10" t="s">
+        <v>152</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -29649,11 +29925,11 @@
     </row>
     <row r="10">
       <c r="A10" s="1"/>
-      <c r="B10" s="9" t="s">
-        <v>9</v>
+      <c r="B10" s="10" t="s">
+        <v>7</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>51</v>
+      <c r="C10" s="10" t="s">
+        <v>153</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -29681,11 +29957,11 @@
     </row>
     <row r="11">
       <c r="A11" s="1"/>
-      <c r="B11" s="9" t="s">
-        <v>10</v>
+      <c r="B11" s="10" t="s">
+        <v>8</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>56</v>
+      <c r="C11" s="10" t="s">
+        <v>154</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -29713,11 +29989,11 @@
     </row>
     <row r="12">
       <c r="A12" s="1"/>
-      <c r="B12" s="9" t="s">
-        <v>12</v>
+      <c r="B12" s="10" t="s">
+        <v>9</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>62</v>
+      <c r="C12" s="10" t="s">
+        <v>155</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -57408,9 +57684,9 @@
       <c r="Z1000" s="1"/>
     </row>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup paperSize="9" scale="68" orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="68" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(scrum): documentar el Sprint 6 y actualizar el seguimiento del proyecto
- Añadir los registros de actividades, horas, seguimiento y retrospectiva del Sprint 6.
- Actualizar los estados, iteraciones y comentarios del Product Backlog.
- Incorporar las horas de los sprints 5 y 6 en la TEC y actualizar los cálculos de costos.
- Ajustar la planificación a siete sprints y documentar la reprogramación en el README de Scrum.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/Documentación/Product Backlog SIGET.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/Documentación/Product Backlog SIGET.xlsx
@@ -1253,29 +1253,45 @@
     </row>
     <row r="5" s="5" customFormat="1" ht="42.75">
       <c r="A5" s="6"/>
-      <c r="B5" s="7" t="s">
-        <v>10</v>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>E1-H1</t>
+        </is>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>11</v>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario de SIGET, necesito iniciar sesión en el sistema mediante el proveedor externo de identidad, con la finalidad de acceder a las funcionalidades autorizadas según mi rol.</t>
+        </is>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>12</v>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Iniciar sesión</t>
+        </is>
       </c>
-      <c r="E5" s="7" t="s">
-        <v>13</v>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>14</v>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>15</v>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>16</v>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>17</v>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Inicio y cierre de sesión implementados y validados manualmente. El acceso aplica los roles y permisos locales.</t>
+        </is>
       </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
@@ -1295,31 +1311,47 @@
       <c r="Y5" s="6"/>
       <c r="Z5" s="6"/>
     </row>
-    <row r="6" s="5" customFormat="1" ht="57">
+    <row r="6" s="5" customFormat="1" ht="57.0">
       <c r="A6" s="6"/>
-      <c r="B6" s="7" t="s">
-        <v>18</v>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>E1-H2</t>
+        </is>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>19</v>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario de SIGET, necesito recuperar el acceso a mi cuenta mediante el proveedor externo de identidad, con la finalidad de restablecer mis credenciales cuando no pueda iniciar sesión.</t>
+        </is>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>20</v>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Recuperar acceso</t>
+        </is>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>13</v>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>21</v>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>2 SP</t>
+        </is>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>15</v>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>22</v>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I6" s="7" t="s">
-        <v>23</v>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Recuperación de acceso implementada y validada manualmente. SIGET no almacena ni modifica contraseñas locales.</t>
+        </is>
       </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
@@ -1339,31 +1371,47 @@
       <c r="Y6" s="6"/>
       <c r="Z6" s="6"/>
     </row>
-    <row r="7" s="5" customFormat="1" ht="57">
+    <row r="7" s="5" customFormat="1" ht="57.0">
       <c r="A7" s="6"/>
-      <c r="B7" s="7" t="s">
-        <v>24</v>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>E1-H3</t>
+        </is>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>25</v>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito gestionar los roles y permisos de los usuarios, con la finalidad de controlar el acceso de los usuarios a las funcionalidades del sistema.</t>
+        </is>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>26</v>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Gestión de roles RBAC</t>
+        </is>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>13</v>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>27</v>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>28</v>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>16</v>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>29</v>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Aprovisionamiento y administración de usuarios, roles y permisos desde PySide6 mediante APIs protegidas. La autorización utiliza los roles y permisos de PostgreSQL.</t>
+        </is>
       </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
@@ -1385,29 +1433,45 @@
     </row>
     <row r="8" s="5" customFormat="1" ht="71.25">
       <c r="A8" s="6"/>
-      <c r="B8" s="7" t="s">
-        <v>30</v>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>E2-H4</t>
+        </is>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>31</v>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito registrar un activo tecnológico en el sistema, con la finalidad de mantener un registro actualizado de los equipos tecnológicos disponibles en la empresa.</t>
+        </is>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>32</v>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Registrar activo TI</t>
+        </is>
       </c>
-      <c r="E8" s="7" t="s">
-        <v>13</v>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>27</v>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G8" s="7" t="s">
-        <v>28</v>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>33</v>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Muy Alta</t>
+        </is>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>34</v>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Registro de activos desde PySide6 mediante API protegida, con validaciones, control de duplicados y persistencia en PostgreSQL.</t>
+        </is>
       </c>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
@@ -1429,29 +1493,45 @@
     </row>
     <row r="9" s="5" customFormat="1" ht="71.25">
       <c r="A9" s="6"/>
-      <c r="B9" s="7" t="s">
-        <v>35</v>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>E2-H5</t>
+        </is>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>36</v>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito modificar la información de un activo tecnológico, con la finalidad de mantener actualizados los datos de los equipos registrados.</t>
+        </is>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>37</v>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Modificar activo TI</t>
+        </is>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>13</v>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>14</v>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>28</v>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H9" s="7" t="s">
-        <v>22</v>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>38</v>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Edición de activos desde PySide6 mediante API protegida. Conserva el código de inventario, valida los campos editables y registra los cambios.</t>
+        </is>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
@@ -1471,31 +1551,47 @@
       <c r="Y9" s="6"/>
       <c r="Z9" s="6"/>
     </row>
-    <row r="10" s="5" customFormat="1" ht="57">
+    <row r="10" s="5" customFormat="1" ht="57.0">
       <c r="A10" s="6"/>
-      <c r="B10" s="7" t="s">
-        <v>39</v>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>E2-H6</t>
+        </is>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>40</v>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito consultar los activos tecnológicos registrados, con la finalidad de conocer la información y estado de los equipos disponibles en la empresa.</t>
+        </is>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>41</v>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Inventario general de activos</t>
+        </is>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>13</v>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>14</v>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G10" s="7" t="s">
-        <v>28</v>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>16</v>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>42</v>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Consulta de inventario desde PySide6 mediante API protegida, con búsqueda y filtros por categoría, ubicación y estado.</t>
+        </is>
       </c>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
@@ -1515,31 +1611,47 @@
       <c r="Y10" s="6"/>
       <c r="Z10" s="6"/>
     </row>
-    <row r="11" s="5" customFormat="1" ht="57">
+    <row r="11" s="5" customFormat="1" ht="57.0">
       <c r="A11" s="6"/>
-      <c r="B11" s="7" t="s">
-        <v>43</v>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>E3-H7</t>
+        </is>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>44</v>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario solicitante, necesito consultar el catálogo de equipos disponibles y registrar una solicitud de asignación por tipo o categoría de equipo, con la finalidad de disponer del equipamiento necesario para realizar mis actividades.</t>
+        </is>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>45</v>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Solicitar asignación de equipo</t>
+        </is>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>13</v>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>27</v>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>28</v>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>33</v>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Muy Alta</t>
+        </is>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>46</v>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Catálogo y formulario Web de solicitud por categoría, con disponibilidad y control de duplicados. El activo físico se selecciona durante la entrega.</t>
+        </is>
       </c>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
@@ -1559,31 +1671,47 @@
       <c r="Y11" s="6"/>
       <c r="Z11" s="6"/>
     </row>
-    <row r="12" s="5" customFormat="1" ht="57">
+    <row r="12" s="5" customFormat="1" ht="57.0">
       <c r="A12" s="6"/>
-      <c r="B12" s="7" t="s">
-        <v>47</v>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>E3-H8</t>
+        </is>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>48</v>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito gestionar las solicitudes de asignación de equipos, con la finalidad de revisar y controlar las solicitudes realizadas por los usuarios.</t>
+        </is>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>49</v>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Aprobación de asignaciones</t>
+        </is>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>13</v>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>27</v>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G12" s="7" t="s">
-        <v>28</v>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>16</v>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I12" s="7" t="s">
-        <v>50</v>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Aprobación o rechazo desde PySide6 por el Administrador, con responsable, fecha, motivo de rechazo y auditoría. La aprobación no reserva un activo físico.</t>
+        </is>
       </c>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
@@ -1603,31 +1731,47 @@
       <c r="Y12" s="6"/>
       <c r="Z12" s="6"/>
     </row>
-    <row r="13" s="5" customFormat="1" ht="57">
+    <row r="13" s="5" customFormat="1" ht="57.0">
       <c r="A13" s="6"/>
-      <c r="B13" s="7" t="s">
-        <v>51</v>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>E3-H9</t>
+        </is>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>52</v>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito consultar las asignaciones de equipos registradas en el sistema, con la finalidad de conocer el estado y la información de las asignaciones realizadas.</t>
+        </is>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>53</v>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Consultar asignaciones</t>
+        </is>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>13</v>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>14</v>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>28</v>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>22</v>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I13" s="7" t="s">
-        <v>54</v>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Consulta de asignaciones activas y finalizadas desde PySide6, con búsqueda por usuario o equipo y filtros por estado.</t>
+        </is>
       </c>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
@@ -1649,29 +1793,45 @@
     </row>
     <row r="14" s="5" customFormat="1" ht="71.25">
       <c r="A14" s="6"/>
-      <c r="B14" s="7" t="s">
-        <v>55</v>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>E3-H20</t>
+        </is>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>56</v>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito registrar la entrega física de un activo compatible con una solicitud de asignación aprobada, con la finalidad de formalizar la asignación y mantener actualizado el estado del activo.</t>
+        </is>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>57</v>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Registrar entrega de equipo</t>
+        </is>
       </c>
-      <c r="E14" s="7" t="s">
-        <v>13</v>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>27</v>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>28</v>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H14" s="7" t="s">
-        <v>33</v>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Muy Alta</t>
+        </is>
       </c>
-      <c r="I14" s="7" t="s">
-        <v>58</v>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>Registro de entrega desde PySide6 de un activo disponible y compatible con una solicitud aprobada. Crea la asignación y actualiza los estados en una transacción. La lectura de códigos corresponde a E8-H19.</t>
+        </is>
       </c>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
@@ -1691,31 +1851,47 @@
       <c r="Y14" s="6"/>
       <c r="Z14" s="6"/>
     </row>
-    <row r="15" s="5" customFormat="1" ht="57">
+    <row r="15" s="5" customFormat="1" ht="57.0">
       <c r="A15" s="6"/>
-      <c r="B15" s="7" t="s">
-        <v>59</v>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>E4-H10</t>
+        </is>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>60</v>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito registrar la devolución de un equipo asignado, con la finalidad de cerrar la asignación y dejar constancia de la recepción física del activo.</t>
+        </is>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>61</v>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Registrar devolución de equipo</t>
+        </is>
       </c>
-      <c r="E15" s="7" t="s">
-        <v>13</v>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>27</v>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>28</v>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H15" s="7" t="s">
-        <v>33</v>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Muy Alta</t>
+        </is>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>62</v>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Recepción y evaluación inicial desde PySide6, con cierre de la asignación, fecha de devolución y técnico responsable.</t>
+        </is>
       </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6"/>
@@ -1737,29 +1913,45 @@
     </row>
     <row r="16" s="5" customFormat="1" ht="71.25">
       <c r="A16" s="6"/>
-      <c r="B16" s="7" t="s">
-        <v>63</v>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>E4-H11</t>
+        </is>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>64</v>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito evaluar y registrar el estado en que se recibe un equipo devuelto, con la finalidad de determinar si puede volver a estar disponible o requiere revisión técnica.</t>
+        </is>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>65</v>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Registrar estado de equipo devuelto</t>
+        </is>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>13</v>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>14</v>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>28</v>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H16" s="7" t="s">
-        <v>16</v>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>66</v>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Evaluación integrada con la devolución. Los equipos operativos quedan Disponibles. Los equipos con daño o falla pasan a En revisión y se genera o asocia un ticket de soporte.</t>
+        </is>
       </c>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
@@ -1779,31 +1971,47 @@
       <c r="Y16" s="6"/>
       <c r="Z16" s="6"/>
     </row>
-    <row r="17" s="5" customFormat="1" ht="57">
+    <row r="17" s="5" customFormat="1" ht="57.0">
       <c r="A17" s="6"/>
-      <c r="B17" s="7" t="s">
-        <v>67</v>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>E5-H13</t>
+        </is>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>68</v>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario solicitante, necesito registrar una solicitud de soporte mediante un ticket, con la finalidad de informar un incidente o solicitar un servicio al área de soporte técnico.</t>
+        </is>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>69</v>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Levantar ticket Service Desk</t>
+        </is>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>13</v>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>27</v>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>28</v>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
       </c>
-      <c r="H17" s="7" t="s">
-        <v>33</v>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Muy Alta</t>
+        </is>
       </c>
-      <c r="I17" s="7" t="s">
-        <v>70</v>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Creación inicial de tickets mediante formulario Web y API, con confirmación, estado inicial, prevención de duplicados y activo opcional autorizado según el rol.</t>
+        </is>
       </c>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
@@ -1823,31 +2031,47 @@
       <c r="Y17" s="6"/>
       <c r="Z17" s="6"/>
     </row>
-    <row r="18" s="5" customFormat="1" ht="57">
+    <row r="18" s="5" customFormat="1" ht="57.0">
       <c r="A18" s="6"/>
-      <c r="B18" s="7" t="s">
-        <v>71</v>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>E4-H12</t>
+        </is>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>72</v>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito consultar el historial de asignaciones, devoluciones y estados de un equipo, con la finalidad de conocer su uso y situación a lo largo del tiempo.</t>
+        </is>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>73</v>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Historial y trazabilidad del equipo</t>
+        </is>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>74</v>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>27</v>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G18" s="7" t="s">
-        <v>75</v>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H18" s="7" t="s">
-        <v>22</v>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>76</v>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>Consulta integrada del historial por equipo desde PySide6. Muestra asignaciones, devoluciones y cambios de estado con fecha, responsable y detalles del movimiento.</t>
+        </is>
       </c>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
@@ -1869,29 +2093,45 @@
     </row>
     <row r="19" s="5" customFormat="1" ht="105.75" customHeight="1">
       <c r="A19" s="6"/>
-      <c r="B19" s="7" t="s">
-        <v>77</v>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>E5-H14</t>
+        </is>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>78</v>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema o Técnico de soporte, necesito gestionar los tickets de soporte según los permisos de mi rol, con la finalidad de asignar responsables, atender las solicitudes y mantener actualizado su estado.</t>
+        </is>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>79</v>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Gestionar tickets de soporte</t>
+        </is>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>74</v>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>27</v>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G19" s="7" t="s">
-        <v>75</v>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H19" s="7" t="s">
-        <v>16</v>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>80</v>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>Gestión de tickets desde API y PySide6: asignación y reasignación administrativas, toma por el Técnico, atención y cambios de estado. Aplica RBAC, seguimiento del SLA y control de concurrencia.</t>
+        </is>
       </c>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
@@ -1913,29 +2153,45 @@
     </row>
     <row r="20" s="5" customFormat="1" ht="42.75">
       <c r="A20" s="6"/>
-      <c r="B20" s="7" t="s">
-        <v>81</v>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>E5-H15</t>
+        </is>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>82</v>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario solicitante, necesito consultar el estado de mis tickets de soporte, con la finalidad de conocer el avance y estado de las solicitudes realizadas.</t>
+        </is>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>83</v>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Seguimiento de tickets</t>
+        </is>
       </c>
-      <c r="E20" s="7" t="s">
-        <v>74</v>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>14</v>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G20" s="7" t="s">
-        <v>75</v>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H20" s="7" t="s">
-        <v>22</v>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>84</v>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>Seguimiento de tickets propios en el portal Web, con listado, detalle, estado, responsable y movimientos registrados durante la atención.</t>
+        </is>
       </c>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
@@ -1957,29 +2213,45 @@
     </row>
     <row r="21" s="5" customFormat="1" ht="99.75">
       <c r="A21" s="6"/>
-      <c r="B21" s="7" t="s">
-        <v>85</v>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>E6-H16</t>
+        </is>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>86</v>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito registrar el diagnóstico y gestionar la orden de trabajo asociada a un ticket, con la finalidad de documentar la falla detectada y la intervención técnica requerida sobre el activo.</t>
+        </is>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>87</v>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Registro de diagnósticos y OT</t>
+        </is>
       </c>
-      <c r="E21" s="7" t="s">
-        <v>74</v>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>88</v>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>8 SP</t>
+        </is>
       </c>
-      <c r="G21" s="7" t="s">
-        <v>75</v>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H21" s="7" t="s">
-        <v>33</v>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Muy Alta</t>
+        </is>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>89</v>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>Registro de diagnósticos y órdenes de trabajo desde PySide6, vinculados al ticket y al activo. Controla el inicio de diagnóstico y reparación, los estados asociados y la atención de tickets activos.</t>
+        </is>
       </c>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
@@ -2001,29 +2273,45 @@
     </row>
     <row r="22" s="5" customFormat="1" ht="71.25">
       <c r="A22" s="6"/>
-      <c r="B22" s="7" t="s">
-        <v>90</v>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>E10-H23</t>
+        </is>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>91</v>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario solicitante, necesito recibir notificaciones por correo sobre el estado de mis solicitudes, con la finalidad de estar informado oportunamente sobre vencimientos o actualizaciones de servicio.</t>
+        </is>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>92</v>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Notificaciones por correo</t>
+        </is>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>74</v>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>14</v>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G22" s="7" t="s">
-        <v>75</v>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H22" s="7" t="s">
-        <v>22</v>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>93</v>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>Envío de correos ante eventos de solicitudes, asignaciones y tickets mediante una API externa. Incluye procesamiento en segundo plano y reintentos. Un fallo de envío no revierte la operación principal.</t>
+        </is>
       </c>
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
@@ -2043,31 +2331,47 @@
       <c r="Y22" s="6"/>
       <c r="Z22" s="6"/>
     </row>
-    <row r="23" s="5" customFormat="1" ht="129.75" customHeight="1">
+    <row r="23" s="5" customFormat="1" ht="71.25" customHeight="1">
       <c r="A23" s="6"/>
-      <c r="B23" s="7" t="s">
-        <v>94</v>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>E6-H24</t>
+        </is>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>95</v>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito pausar una orden de trabajo por espera de repuestos o reasignarla a otro Técnico de soporte, con la finalidad de transparentar los cuellos de botella y mantener correctamente registrada la medición del tiempo de resolución (SLA).</t>
+        </is>
       </c>
-      <c r="D23" s="7" t="s">
-        <v>96</v>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Pausa o derivación de OT</t>
+        </is>
       </c>
-      <c r="E23" s="7" t="s">
-        <v>74</v>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>27</v>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>97</v>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H23" s="7" t="s">
-        <v>16</v>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>98</v>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>Pausa, reanudación y reasignación de órdenes de trabajo desde PySide6. Conserva la fase técnica al reanudar y registra motivos, responsables y tiempos para la trazabilidad y el SLA.</t>
+        </is>
       </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
@@ -2089,29 +2393,45 @@
     </row>
     <row r="24" s="5" customFormat="1" ht="71.25">
       <c r="A24" s="6"/>
-      <c r="B24" s="7" t="s">
-        <v>99</v>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>E9-H22</t>
+        </is>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>100</v>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito consultar el registro histórico de operaciones y eventos críticos, con la finalidad de auditar las acciones realizadas sobre los activos y solicitudes.</t>
+        </is>
       </c>
-      <c r="D24" s="7" t="s">
-        <v>101</v>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Bitácora de auditoría</t>
+        </is>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>74</v>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>14</v>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G24" s="7" t="s">
-        <v>97</v>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H24" s="7" t="s">
-        <v>22</v>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I24" s="7" t="s">
-        <v>102</v>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>Consulta de auditoría desde PySide6 con búsqueda y filtros por actor, recurso, módulo, acción y fecha. Acceso de Administrador y registros protegidos contra edición y eliminación.</t>
+        </is>
       </c>
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
@@ -2131,31 +2451,47 @@
       <c r="Y24" s="6"/>
       <c r="Z24" s="6"/>
     </row>
-    <row r="25" s="5" customFormat="1" ht="42.75">
+    <row r="25" s="5" customFormat="1" ht="57.0">
       <c r="A25" s="6"/>
-      <c r="B25" s="7" t="s">
-        <v>103</v>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>E10-H29</t>
+        </is>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>104</v>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario solicitante, necesito visualizar un centro de notificaciones dentro de la plataforma, con la finalidad de enterarme de avisos urgentes aunque no revise mi correo electrónico.</t>
+        </is>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>105</v>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Centro de avisos en plataforma</t>
+        </is>
       </c>
-      <c r="E25" s="7" t="s">
-        <v>74</v>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>27</v>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G25" s="7" t="s">
-        <v>97</v>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H25" s="7" t="s">
-        <v>22</v>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I25" s="7" t="s">
-        <v>106</v>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Bandeja de notificaciones del solicitante con contador de avisos sin leer, detalle del mensaje y acceso al recurso asociado. La apertura desde la bandeja marca el aviso como leído.</t>
+        </is>
       </c>
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
@@ -2175,31 +2511,47 @@
       <c r="Y25" s="6"/>
       <c r="Z25" s="6"/>
     </row>
-    <row r="26" s="5" customFormat="1" ht="42.75">
+    <row r="26" s="5" customFormat="1" ht="57.0">
       <c r="A26" s="6"/>
-      <c r="B26" s="7" t="s">
-        <v>107</v>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>E5-H30</t>
+        </is>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>108</v>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Como un Usuario solicitante, necesito calificar la atención recibida al cerrarse un ticket de soporte, con la finalidad de aportar retroalimentación sobre la calidad del servicio técnico.</t>
+        </is>
       </c>
-      <c r="D26" s="7" t="s">
-        <v>109</v>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Calificación de servicio (CSAT)</t>
+        </is>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>74</v>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>14</v>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G26" s="7" t="s">
-        <v>97</v>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
       </c>
-      <c r="H26" s="7" t="s">
-        <v>22</v>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I26" s="7" t="s">
-        <v>110</v>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Calificación de la atención desde el portal Web para tickets propios cerrados. Permite registrar una evaluación y un comentario, con control de acceso y prevención de calificaciones duplicadas.</t>
+        </is>
       </c>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
@@ -2219,31 +2571,47 @@
       <c r="Y26" s="6"/>
       <c r="Z26" s="6"/>
     </row>
-    <row r="27" s="5" customFormat="1" ht="57">
+    <row r="27" s="5" customFormat="1" ht="129.75">
       <c r="A27" s="6"/>
-      <c r="B27" s="7" t="s">
-        <v>111</v>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>E6-H17</t>
+        </is>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>112</v>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito registrar el cierre y resolución de una reparación, con la finalidad de certificar la operatividad del equipo para que vuelva a estar disponible.</t>
+        </is>
       </c>
-      <c r="D27" s="7" t="s">
-        <v>113</v>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Cierre técnico de reparación</t>
+        </is>
       </c>
-      <c r="E27" s="7" t="s">
-        <v>74</v>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>14</v>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G27" s="7" t="s">
-        <v>97</v>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H27" s="7" t="s">
-        <v>22</v>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I27" s="7" t="s">
-        <v>114</v>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Cierra la OT y resuelve el ticket con el resultado técnico registrado. Si la reparación finaliza con éxito, el activo vuelve a Disponible. Si es no reparable, exige informe de descarte, completa la OT, deja el activo Dado de baja, resuelve el ticket y notifica al administrador de inventario. El ticket se cierra posteriormente mediante su flujo habitual.</t>
+        </is>
       </c>
       <c r="J27" s="6"/>
       <c r="K27" s="6"/>
@@ -2263,31 +2631,47 @@
       <c r="Y27" s="6"/>
       <c r="Z27" s="6"/>
     </row>
-    <row r="28" s="5" customFormat="1" ht="71.25">
+    <row r="28" s="5" customFormat="1" ht="42.75">
       <c r="A28" s="6"/>
-      <c r="B28" s="7" t="s">
-        <v>115</v>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>E7-H18</t>
+        </is>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>116</v>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito registrar los repuestos utilizados en una reparación, con la finalidad de descontar el stock utilizado y mantener el control de piezas de recambio.</t>
+        </is>
       </c>
-      <c r="D28" s="7" t="s">
-        <v>117</v>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Asignación de repuestos</t>
+        </is>
       </c>
-      <c r="E28" s="7" t="s">
-        <v>74</v>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>27</v>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>97</v>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H28" s="7" t="s">
-        <v>16</v>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I28" s="7" t="s">
-        <v>118</v>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Imputación de repuestos a órdenes de trabajo y actualización transaccional de existencias.</t>
+        </is>
       </c>
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
@@ -2307,31 +2691,47 @@
       <c r="Y28" s="6"/>
       <c r="Z28" s="6"/>
     </row>
-    <row r="29" s="5" customFormat="1" ht="71.25">
+    <row r="29" s="5" customFormat="1" ht="57.0">
       <c r="A29" s="6"/>
-      <c r="B29" s="7" t="s">
-        <v>119</v>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>E7-H25</t>
+        </is>
       </c>
-      <c r="C29" s="7" t="s">
-        <v>120</v>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito registrar el ingreso y compra de nuevos repuestos, con la finalidad de mantener abastecido el inventario de piezas para reparaciones.</t>
+        </is>
       </c>
-      <c r="D29" s="7" t="s">
-        <v>121</v>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Carga de stock de repuestos</t>
+        </is>
       </c>
-      <c r="E29" s="7" t="s">
-        <v>74</v>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>27</v>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G29" s="7" t="s">
-        <v>122</v>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H29" s="7" t="s">
-        <v>22</v>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>123</v>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Administración de repuestos y registro de ingresos de stock desde PySide6 mediante API protegida. Registra compras, existencias y movimientos de inventario con persistencia en PostgreSQL.</t>
+        </is>
       </c>
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
@@ -2351,31 +2751,47 @@
       <c r="Y29" s="6"/>
       <c r="Z29" s="6"/>
     </row>
-    <row r="30" s="5" customFormat="1" ht="57">
+    <row r="30" s="5" customFormat="1" ht="57.0">
       <c r="A30" s="6"/>
-      <c r="B30" s="7" t="s">
-        <v>124</v>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>E7-H26</t>
+        </is>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>125</v>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito visualizar alertas automáticas ante repuestos bajo el stock mínimo, con la finalidad de gestionar oportunamente las adquisiciones y evitar quiebres en taller.</t>
+        </is>
       </c>
-      <c r="D30" s="7" t="s">
-        <v>126</v>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Alerta de stock crítico</t>
+        </is>
       </c>
-      <c r="E30" s="7" t="s">
-        <v>74</v>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>27</v>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G30" s="7" t="s">
-        <v>122</v>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H30" s="7" t="s">
-        <v>22</v>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I30" s="7" t="s">
-        <v>127</v>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>Alertas de repuestos bajo el mínimo configurado y ajuste de existencias desde PySide6, con autorización de Administrador, validaciones y registro de los movimientos.</t>
+        </is>
       </c>
       <c r="J30" s="6"/>
       <c r="K30" s="6"/>
@@ -2397,29 +2813,45 @@
     </row>
     <row r="31" s="5" customFormat="1" ht="71.25">
       <c r="A31" s="6"/>
-      <c r="B31" s="7" t="s">
-        <v>128</v>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>E8-H19</t>
+        </is>
       </c>
-      <c r="C31" s="7" t="s">
-        <v>129</v>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Como un Técnico de soporte, necesito leer códigos de barra o QR de los equipos, con la finalidad de identificar con precisión los activos durante su entrega, devolución y operación técnica.</t>
+        </is>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>130</v>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Lectura de códigos QR/Barras</t>
+        </is>
       </c>
-      <c r="E31" s="7" t="s">
-        <v>74</v>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>14</v>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G31" s="7" t="s">
-        <v>122</v>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H31" s="7" t="s">
-        <v>22</v>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
       </c>
-      <c r="I31" s="7" t="s">
-        <v>131</v>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>Lectura local mediante lector físico USB HID en PySide6, principalmente durante los procesos de entrega y devolución. Esta lectura no se contabiliza como una API externa, conforme a RNF19.</t>
+        </is>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
@@ -2439,31 +2871,47 @@
       <c r="Y31" s="6"/>
       <c r="Z31" s="6"/>
     </row>
-    <row r="32" s="5" customFormat="1" ht="42.75">
+    <row r="32" s="5" customFormat="1" ht="71.25">
       <c r="A32" s="6"/>
-      <c r="B32" s="7" t="s">
-        <v>132</v>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>E8-H27</t>
+        </is>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>133</v>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito generar e imprimir etiquetas con código QR para activos nuevos, con la finalidad de rotular físicamente los equipos que ingresan a la flota institucional.</t>
+        </is>
       </c>
-      <c r="D32" s="7" t="s">
-        <v>134</v>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Generación de códigos QR</t>
+        </is>
       </c>
-      <c r="E32" s="7" t="s">
-        <v>74</v>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
       </c>
-      <c r="F32" s="7" t="s">
-        <v>14</v>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G32" s="7" t="s">
-        <v>122</v>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H32" s="7" t="s">
-        <v>22</v>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I32" s="7" t="s">
-        <v>135</v>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t>Generación de códigos QR mediante la API externa definida para SIGET, asociándolos al activo correspondiente; impresión y reimpresión de etiquetas desde la aplicación de Escritorio.</t>
+        </is>
       </c>
       <c r="J32" s="6"/>
       <c r="K32" s="6"/>
@@ -2483,31 +2931,47 @@
       <c r="Y32" s="6"/>
       <c r="Z32" s="6"/>
     </row>
-    <row r="33" s="5" customFormat="1" ht="57">
+    <row r="33" s="5" customFormat="1" ht="57.0">
       <c r="A33" s="6"/>
-      <c r="B33" s="7" t="s">
-        <v>136</v>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>E9-H21</t>
+        </is>
       </c>
-      <c r="C33" s="7" t="s">
-        <v>137</v>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito consultar reportes de fallas y tiempos de atención, con la finalidad de evaluar el rendimiento del servicio y apoyar la toma de decisiones sobre el parque tecnológico.</t>
+        </is>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>138</v>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Reportes y métricas de soporte</t>
+        </is>
       </c>
-      <c r="E33" s="7" t="s">
-        <v>74</v>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>14</v>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>5 SP</t>
+        </is>
       </c>
-      <c r="G33" s="7" t="s">
-        <v>122</v>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H33" s="7" t="s">
-        <v>22</v>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I33" s="7" t="s">
-        <v>139</v>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>Métricas de SLA, tiempos de atención y recurrencia de fallas basadas en datos históricos.</t>
+        </is>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
@@ -2529,29 +2993,45 @@
     </row>
     <row r="34" s="5" customFormat="1" ht="42.75">
       <c r="A34" s="6"/>
-      <c r="B34" s="7" t="s">
-        <v>140</v>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>E9-H28</t>
+        </is>
       </c>
-      <c r="C34" s="7" t="s">
-        <v>141</v>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Como un Administrador del sistema, necesito exportar informes ejecutivos del estado y valorización del parque tecnológico, con la finalidad de respaldar auditorías contables e inversiones de TI.</t>
+        </is>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>142</v>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Reporte consolidado de parque TI</t>
+        </is>
       </c>
-      <c r="E34" s="7" t="s">
-        <v>74</v>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Planificada</t>
+        </is>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>14</v>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>3 SP</t>
+        </is>
       </c>
-      <c r="G34" s="7" t="s">
-        <v>122</v>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 7</t>
+        </is>
       </c>
-      <c r="H34" s="7" t="s">
-        <v>22</v>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
       </c>
-      <c r="I34" s="7" t="s">
-        <v>143</v>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t>Generación de informes consolidados y exportación a PDF/Excel.</t>
+        </is>
       </c>
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>

</xml_diff>